<commit_message>
Refactor feature scaling and vector operations
- Replaced Standardiser with new EuclidianScaler, MinMaxScaler, and ZScoreScaler, all implementing a simplified IFeatureScaler for vector-based scaling
- Refactored Vector from class to struct, added scaling methods, operator overloads, and improved magnitude/equality logic
- Introduced parser infrastructure for string-to-vector conversion with tests
- Updated and expanded unit tests for all new and existing vector and scaler functionality
- Cleaned up error function provider interface and improved documentation
- Modernized test setup (Moq, ITestOutputHelper injection, copyright)
- Marked legacy code as excluded from coverage
- Updated project files and feature scaling checker Excel file
</commit_message>
<xml_diff>
--- a/NeuralNetworks.Test/FeatureScaling/feature scaling checker.xlsx
+++ b/NeuralNetworks.Test/FeatureScaling/feature scaling checker.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simon\source\repos\NeuralNetworks\NeuralNetworks.Test\FeatureScaling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DA435C2-F28F-4442-A120-259884D564CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{07E7C126-AF57-40D5-95AB-3CDA9D6367A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-56385" yWindow="-390" windowWidth="26865" windowHeight="11295" xr2:uid="{312A9268-7947-4495-9E35-DA32BA9258CD}"/>
+    <workbookView xWindow="-55860" yWindow="30" windowWidth="26865" windowHeight="11295" activeTab="2" xr2:uid="{312A9268-7947-4495-9E35-DA32BA9258CD}"/>
   </bookViews>
   <sheets>
-    <sheet name="Standardisation and stdDev" sheetId="1" r:id="rId1"/>
+    <sheet name="z-score and stdDev" sheetId="1" r:id="rId1"/>
+    <sheet name="Euclidian" sheetId="2" r:id="rId2"/>
+    <sheet name="Min-max" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="20">
   <si>
     <t>Feature 1</t>
   </si>
@@ -69,6 +72,33 @@
   </si>
   <si>
     <t>Standardised using sample stdDev</t>
+  </si>
+  <si>
+    <t>Record 4</t>
+  </si>
+  <si>
+    <t>Scaled</t>
+  </si>
+  <si>
+    <t>Euclidian magnitudes</t>
+  </si>
+  <si>
+    <t>Squared values</t>
+  </si>
+  <si>
+    <t>Scaled Euclidean magnitudes</t>
+  </si>
+  <si>
+    <t>Scaled squared</t>
+  </si>
+  <si>
+    <t>Minimum values</t>
+  </si>
+  <si>
+    <t>Maximum values</t>
+  </si>
+  <si>
+    <t>Scaled values</t>
   </si>
 </sst>
 </file>
@@ -119,19 +149,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -466,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B2D1460-73F1-443A-AEFD-30ECC48B42F1}">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="4.42578125" customWidth="1"/>
@@ -479,158 +511,184 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="E1" s="5" t="s">
+      <c r="C1" s="3"/>
+      <c r="E1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="5"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="5" t="s">
+      <c r="F1" s="4"/>
+      <c r="H1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="5"/>
+      <c r="I1" s="4"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="M2" s="4" t="s">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="4">
-        <v>0</v>
-      </c>
-      <c r="C3" s="4">
-        <v>400</v>
-      </c>
-      <c r="E3" s="4">
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2">
+        <v>6</v>
+      </c>
+      <c r="E3" s="2">
+        <f>STANDARDIZE(B3,L$3,L$4)</f>
+        <v>-1.3055824196677337</v>
+      </c>
+      <c r="F3" s="2">
+        <f>STANDARDIZE(C3,M$3,M$4)</f>
+        <v>0.9209401941068136</v>
+      </c>
+      <c r="H3" s="2">
         <f>STANDARDIZE(B3,L$3,L$5)</f>
-        <v>-0.836357190572102</v>
-      </c>
-      <c r="F3" s="4">
+        <v>-1.507556722888818</v>
+      </c>
+      <c r="I3" s="2">
         <f>STANDARDIZE(C3,M$3,M$5)</f>
-        <v>1.413451334921205</v>
-      </c>
-      <c r="H3" s="4">
-        <f>STANDARDIZE(E3,L$3,L$5)</f>
-        <v>-0.88100570228837816</v>
-      </c>
-      <c r="I3" s="4">
-        <f>STANDARDIZE(F3,M$3,M$5)</f>
-        <v>-0.72327188616207505</v>
-      </c>
-      <c r="K3" s="4" t="s">
+        <v>1.0634101379502299</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="2">
         <f>AVERAGE(B:B)</f>
-        <v>15.666666666666666</v>
-      </c>
-      <c r="M3" s="4">
+        <v>3.5</v>
+      </c>
+      <c r="M3" s="2">
         <f>AVERAGE(C:C)</f>
-        <v>136.33333333333334</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4">
-        <v>42</v>
-      </c>
-      <c r="C4" s="4">
-        <v>-3</v>
-      </c>
-      <c r="E4" s="4">
-        <f>STANDARDIZE(B4,L$3,L$5)</f>
-        <v>1.4057918735148098</v>
-      </c>
-      <c r="F4" s="4">
-        <f>STANDARDIZE(C4,M$3,M$5)</f>
-        <v>-0.74693129961702132</v>
-      </c>
-      <c r="H4" s="4">
-        <f t="shared" ref="H4:H5" si="0">STANDARDIZE(E4,L$3,L$5)</f>
-        <v>-0.76130969215538247</v>
-      </c>
-      <c r="I4" s="4">
-        <f t="shared" ref="I4:I5" si="1">STANDARDIZE(F4,M$3,M$5)</f>
-        <v>-0.73485315943158946</v>
-      </c>
-      <c r="K4" s="4" t="s">
+      <c r="B4" s="2">
         <v>5</v>
       </c>
-      <c r="L4" s="4">
+      <c r="C4" s="2">
+        <v>-1</v>
+      </c>
+      <c r="E4" s="2">
+        <f t="shared" ref="E4:E6" si="0">STANDARDIZE(B4,L$3,L$4)</f>
+        <v>0.78334945180064031</v>
+      </c>
+      <c r="F4" s="2">
+        <f t="shared" ref="F4:F6" si="1">STANDARDIZE(C4,M$3,M$4)</f>
+        <v>-1.4232712090741664</v>
+      </c>
+      <c r="H4" s="2">
+        <f t="shared" ref="H4:H6" si="2">STANDARDIZE(B4,L$3,L$5)</f>
+        <v>0.90453403373329089</v>
+      </c>
+      <c r="I4" s="2">
+        <f t="shared" ref="I4:I6" si="3">STANDARDIZE(C4,M$3,M$5)</f>
+        <v>-1.643452031377628</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L4" s="2">
         <f>_xlfn.STDEV.S(B:B)</f>
-        <v>22.941955743426348</v>
-      </c>
-      <c r="M4" s="4">
+        <v>1.9148542155126762</v>
+      </c>
+      <c r="M4" s="2">
         <f>_xlfn.STDEV.S(C:C)</f>
-        <v>228.46516875299247</v>
+        <v>2.9860788111948193</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="2">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2">
+        <f t="shared" si="0"/>
+        <v>-0.26111648393354675</v>
+      </c>
+      <c r="F5" s="2">
+        <f t="shared" si="1"/>
+        <v>0.25116550748367644</v>
+      </c>
+      <c r="H5" s="2">
+        <f t="shared" si="2"/>
+        <v>-0.30151134457776363</v>
+      </c>
+      <c r="I5" s="2">
+        <f t="shared" si="3"/>
+        <v>0.29002094671369905</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="L5" s="2">
+        <f>_xlfn.STDEV.P(B:B)</f>
+        <v>1.6583123951776999</v>
+      </c>
+      <c r="M5" s="2">
+        <f>_xlfn.STDEV.P(C:C)</f>
+        <v>2.5860201081971503</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="2">
         <v>5</v>
       </c>
-      <c r="C5" s="4">
-        <v>12</v>
-      </c>
-      <c r="E5" s="4">
-        <f>STANDARDIZE(B5,L$3,L$5)</f>
-        <v>-0.56943468294270772</v>
-      </c>
-      <c r="F5" s="4">
-        <f>STANDARDIZE(C5,M$3,M$5)</f>
-        <v>-0.66652003530418402</v>
-      </c>
-      <c r="H5" s="4">
+      <c r="C6" s="2">
+        <v>4</v>
+      </c>
+      <c r="E6" s="2">
         <f t="shared" si="0"/>
-        <v>-0.86675617727254528</v>
-      </c>
-      <c r="I5" s="4">
+        <v>0.78334945180064031</v>
+      </c>
+      <c r="F6" s="2">
         <f t="shared" si="1"/>
-        <v>-0.73442209466969699</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="L5" s="4">
-        <f>_xlfn.STDEV.P(B:B)</f>
-        <v>18.732028424302822</v>
-      </c>
-      <c r="M5" s="4">
-        <f>_xlfn.STDEV.P(C:C)</f>
-        <v>186.54102914789431</v>
+        <v>0.25116550748367644</v>
+      </c>
+      <c r="H6" s="2">
+        <f t="shared" si="2"/>
+        <v>0.90453403373329089</v>
+      </c>
+      <c r="I6" s="2">
+        <f t="shared" si="3"/>
+        <v>0.29002094671369905</v>
       </c>
     </row>
   </sheetData>
@@ -641,4 +699,380 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B39FC3B-C99D-417D-8DD4-F85413747D5F}">
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="5"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="6"/>
+      <c r="H1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L2" t="s">
+        <v>1</v>
+      </c>
+      <c r="N2" t="s">
+        <v>0</v>
+      </c>
+      <c r="O2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>0</v>
+      </c>
+      <c r="R2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>-23</v>
+      </c>
+      <c r="E3">
+        <f>POWER(B3,2)</f>
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <f>POWER(C3,2)</f>
+        <v>529</v>
+      </c>
+      <c r="H3" s="7">
+        <f>SUM(E:E)</f>
+        <v>30</v>
+      </c>
+      <c r="I3" s="7">
+        <f>SUM(F:F)</f>
+        <v>3654.04</v>
+      </c>
+      <c r="K3">
+        <f>B3/H$3</f>
+        <v>3.3333333333333333E-2</v>
+      </c>
+      <c r="L3">
+        <f>C3/I$3</f>
+        <v>-6.2944029074668041E-3</v>
+      </c>
+      <c r="N3">
+        <f>POWER(K3,2)</f>
+        <v>1.1111111111111111E-3</v>
+      </c>
+      <c r="O3">
+        <f>POWER(L3,2)</f>
+        <v>3.9619507961526555E-5</v>
+      </c>
+      <c r="Q3">
+        <f>SQRT(SUM(N:N))</f>
+        <v>0.18257418583505539</v>
+      </c>
+      <c r="R3">
+        <f>SQRT(SUM(O:O))</f>
+        <v>1.6542965019276063E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>55</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:F6" si="0">POWER(B4,2)</f>
+        <v>4</v>
+      </c>
+      <c r="F4">
+        <f>POWER(C4,2)</f>
+        <v>3025</v>
+      </c>
+      <c r="K4">
+        <f>B4/H$3</f>
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="L4">
+        <f>C4/I$3</f>
+        <v>1.5051833039594531E-2</v>
+      </c>
+      <c r="N4">
+        <f t="shared" ref="N4:N6" si="1">POWER(K4,2)</f>
+        <v>4.4444444444444444E-3</v>
+      </c>
+      <c r="O4">
+        <f t="shared" ref="O4:O6" si="2">POWER(L4,2)</f>
+        <v>2.2655767785182955E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>0.2</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>4.0000000000000008E-2</v>
+      </c>
+      <c r="K5">
+        <f>B5/H$3</f>
+        <v>0.1</v>
+      </c>
+      <c r="L5">
+        <f>C5/I$3</f>
+        <v>5.4733938325798299E-5</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="1"/>
+        <v>1.0000000000000002E-2</v>
+      </c>
+      <c r="O5">
+        <f t="shared" si="2"/>
+        <v>2.995804004652292E-9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>-10</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="K6">
+        <f>B6/H$3</f>
+        <v>0.13333333333333333</v>
+      </c>
+      <c r="L6">
+        <f>C6/I$3</f>
+        <v>-2.7366969162899149E-3</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="1"/>
+        <v>1.7777777777777778E-2</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="2"/>
+        <v>7.4895100116307296E-6</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67CE0858-7ECF-43D3-8DE4-323BA3D29D5E}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>-23</v>
+      </c>
+      <c r="E3">
+        <f>MIN(B:B)</f>
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <f>MIN(C:C)</f>
+        <v>-23</v>
+      </c>
+      <c r="G3">
+        <f>MAX(B:B)</f>
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <f>MAX(C:C)</f>
+        <v>55</v>
+      </c>
+      <c r="J3">
+        <f>(B3-E$3)/(G$3-E$3)</f>
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <f>(C3-F$3)/(H$3-F$3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>55</v>
+      </c>
+      <c r="J4">
+        <f t="shared" ref="J4:J6" si="0">(B4-E$3)/(G$3-E$3)</f>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="K4">
+        <f t="shared" ref="K4:K6" si="1">(C4-F$3)/(H$3-F$3)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>0.2</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="0"/>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="1"/>
+        <v>0.29743589743589743</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>-10</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="1"/>
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Matrix <--> string two-way conversion and unit tests
</commit_message>
<xml_diff>
--- a/NeuralNetworks.Test/FeatureScaling/feature scaling checker.xlsx
+++ b/NeuralNetworks.Test/FeatureScaling/feature scaling checker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simon\source\repos\NeuralNetworks\NeuralNetworks.Test\FeatureScaling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{07E7C126-AF57-40D5-95AB-3CDA9D6367A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{695B0A01-A390-41F4-A6A8-BF1C8E42AB17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-55860" yWindow="30" windowWidth="26865" windowHeight="11295" activeTab="2" xr2:uid="{312A9268-7947-4495-9E35-DA32BA9258CD}"/>
+    <workbookView xWindow="-55860" yWindow="30" windowWidth="19350" windowHeight="11295" activeTab="1" xr2:uid="{312A9268-7947-4495-9E35-DA32BA9258CD}"/>
   </bookViews>
   <sheets>
     <sheet name="z-score and stdDev" sheetId="1" r:id="rId1"/>
@@ -790,36 +790,36 @@
         <v>529</v>
       </c>
       <c r="H3" s="7">
-        <f>SUM(E:E)</f>
-        <v>30</v>
+        <f>SQRT(SUM(E:E))</f>
+        <v>5.4772255750516612</v>
       </c>
       <c r="I3" s="7">
-        <f>SUM(F:F)</f>
-        <v>3654.04</v>
+        <f>SQRT(SUM(F:F))</f>
+        <v>60.448655899035508</v>
       </c>
       <c r="K3">
         <f>B3/H$3</f>
-        <v>3.3333333333333333E-2</v>
+        <v>0.18257418583505536</v>
       </c>
       <c r="L3">
         <f>C3/I$3</f>
-        <v>-6.2944029074668041E-3</v>
+        <v>-0.38048819544334944</v>
       </c>
       <c r="N3">
         <f>POWER(K3,2)</f>
-        <v>1.1111111111111111E-3</v>
+        <v>3.3333333333333326E-2</v>
       </c>
       <c r="O3">
         <f>POWER(L3,2)</f>
-        <v>3.9619507961526555E-5</v>
+        <v>0.14477126687173647</v>
       </c>
       <c r="Q3">
         <f>SQRT(SUM(N:N))</f>
-        <v>0.18257418583505539</v>
+        <v>0.99999999999999989</v>
       </c>
       <c r="R3">
         <f>SQRT(SUM(O:O))</f>
-        <v>1.6542965019276063E-2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -842,19 +842,19 @@
       </c>
       <c r="K4">
         <f>B4/H$3</f>
-        <v>6.6666666666666666E-2</v>
+        <v>0.36514837167011072</v>
       </c>
       <c r="L4">
         <f>C4/I$3</f>
-        <v>1.5051833039594531E-2</v>
+        <v>0.90986307606018346</v>
       </c>
       <c r="N4">
         <f t="shared" ref="N4:N6" si="1">POWER(K4,2)</f>
-        <v>4.4444444444444444E-3</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="O4">
         <f t="shared" ref="O4:O6" si="2">POWER(L4,2)</f>
-        <v>2.2655767785182955E-4</v>
+        <v>0.82785081717769915</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -877,19 +877,19 @@
       </c>
       <c r="K5">
         <f>B5/H$3</f>
-        <v>0.1</v>
+        <v>0.54772255750516607</v>
       </c>
       <c r="L5">
         <f>C5/I$3</f>
-        <v>5.4733938325798299E-5</v>
+        <v>3.3085930038552125E-3</v>
       </c>
       <c r="N5">
         <f t="shared" si="1"/>
-        <v>1.0000000000000002E-2</v>
+        <v>0.29999999999999993</v>
       </c>
       <c r="O5">
         <f t="shared" si="2"/>
-        <v>2.995804004652292E-9</v>
+        <v>1.0946787665159659E-5</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -912,19 +912,19 @@
       </c>
       <c r="K6">
         <f>B6/H$3</f>
-        <v>0.13333333333333333</v>
+        <v>0.73029674334022143</v>
       </c>
       <c r="L6">
         <f>C6/I$3</f>
-        <v>-2.7366969162899149E-3</v>
+        <v>-0.16542965019276062</v>
       </c>
       <c r="N6">
         <f t="shared" si="1"/>
-        <v>1.7777777777777778E-2</v>
+        <v>0.53333333333333321</v>
       </c>
       <c r="O6">
         <f t="shared" si="2"/>
-        <v>7.4895100116307296E-6</v>
+        <v>2.7366969162899147E-2</v>
       </c>
     </row>
   </sheetData>
@@ -939,6 +939,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67CE0858-7ECF-43D3-8DE4-323BA3D29D5E}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="10" max="10" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
@@ -1049,7 +1053,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="K5">
-        <f t="shared" si="1"/>
+        <f>(C5-F$3)/(H$3-F$3)</f>
         <v>0.29743589743589743</v>
       </c>
     </row>

</xml_diff>